<commit_message>
commited on 9 nov
</commit_message>
<xml_diff>
--- a/assets/files/heads.xlsx
+++ b/assets/files/heads.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\iism\assets\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C06E292-3F0A-451E-BC5D-1F2A92BDC645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D3BBE7-EA7E-483B-9DF3-4DC1E72EEF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="61">
   <si>
     <t>Position</t>
   </si>
@@ -197,13 +197,19 @@
   </si>
   <si>
     <t>Head , Finance</t>
+  </si>
+  <si>
+    <t>Aakansh Chandra</t>
+  </si>
+  <si>
+    <t>aakanshc21@iitk.ac.in</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -226,6 +232,13 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -257,10 +270,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -277,8 +291,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -495,7 +519,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U23"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
@@ -504,7 +528,7 @@
     <col min="4" max="4" width="19.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -518,7 +542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -532,7 +556,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -546,7 +570,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>57</v>
       </c>
@@ -560,7 +584,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>57</v>
       </c>
@@ -574,7 +598,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
@@ -588,7 +612,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>33</v>
       </c>
@@ -602,7 +626,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>33</v>
       </c>
@@ -616,230 +640,243 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="6">
+        <v>210007</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="7"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C10" s="4">
         <v>210597</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="2">
-        <v>210655</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="2">
+        <v>210655</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C12" s="2">
         <v>210593</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2">
-        <v>211085</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="2">
+        <v>211085</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C14" s="2">
         <v>210664</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="2">
-        <v>210893</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="2">
+        <v>210893</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C16" s="2">
         <v>210749</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="2">
-        <v>210985</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="C17" s="2">
-        <v>210673</v>
+        <v>210985</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="2">
+        <v>210673</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C19" s="2">
         <v>210467</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C20" s="2">
         <v>210754</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5"/>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
-      <c r="U19" s="5"/>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="2">
-        <v>210764</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5"/>
+      <c r="S20" s="5"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="2">
+        <v>210764</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C22" s="2">
         <v>210678</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C23" s="3">
         <v>221015</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C24" s="2">
         <v>220921</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -847,6 +884,9 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D24">
     <sortCondition descending="1" ref="A1:A24"/>
   </sortState>
+  <hyperlinks>
+    <hyperlink ref="D9" r:id="rId1" xr:uid="{157A682D-DF24-4B87-B806-A7F198D9BD75}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>